<commit_message>
Build Investment Services OA V01 from reassembled OA
</commit_message>
<xml_diff>
--- a/Project Rooms/Operating Agreements/working/Investment Services/Investment Services OA Process Control.xlsx
+++ b/Project Rooms/Operating Agreements/working/Investment Services/Investment Services OA Process Control.xlsx
@@ -6385,7 +6385,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -6512,7 +6511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z200"/>
+  <dimension ref="A1:Z201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.75" customWidth="1" min="1" max="1"/>
@@ -6532,6 +6531,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -12148,6 +12148,43 @@
       <c r="Y200" s="5" t="n"/>
       <c r="Z200" s="5" t="n"/>
     </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>IS V01</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>IS V01 - Investment Services OA Draft - from Reassembled OA Check.docx</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Reassembled OA Check / SYH framework</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>First Investment Services draft. Redlines SYH entity name to Investment Services LLC, strikes opening retirement-account member lines, inserts Investment Services member placeholder, marks Manager(s), tax classification, certification/signature, and Exhibit A as unconfirmed.</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>Structural DOCX checks passed. Visual render not completed because converter path was unavailable.</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Open facts: members/ownership, managers, tax classification, effective date, signer titles, Exhibit A.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
@@ -12162,7 +12199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z214"/>
+  <dimension ref="A1:Z216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12182,6 +12219,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -18153,6 +18191,70 @@
       <c r="F214" s="14" t="n"/>
       <c r="G214" s="14" t="n"/>
       <c r="H214" s="14" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>IS-START-REASSEMBLED</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Source selection</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>All Investment Services drafts using the SYH/Simplified OA framework begin from the Reassembled OA Check unless Wes explicitly names another source.</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Wes instruction 2026-06-16</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Applied in IS V01</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>IS-NO-WYOMING-SOURCE</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Source exclusion</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Do not use the Wyoming Investment Services OA as the drafting source unless Wes explicitly changes that rule.</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Wes instruction 2026-06-16</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Applied in IS V01</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -24325,7 +24427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z200"/>
+  <dimension ref="A1:Z203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.25" customWidth="1" min="1" max="1"/>
@@ -24345,6 +24447,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -30145,6 +30248,102 @@
       <c r="Y200" s="5" t="n"/>
       <c r="Z200" s="5" t="n"/>
     </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>IS-MEMBERS</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Member facts</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Confirm current Investment Services LLC member(s), ownership units or percentages, contributions, and whether any retirement-account ownership exists.</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Wes/records</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>IS-MANAGERS</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Manager facts</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Confirm current Investment Services LLC manager(s) and signer titles.</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Wes/records</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>IS-TAX</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Tax classification</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Confirm tax classification before finalizing pass-through, S-corp, IRA, UBTI/UDFI, or retirement-account provisions.</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>CPA/attorney</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
@@ -30159,7 +30358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z209"/>
+  <dimension ref="A1:Z210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.75" customWidth="1" min="1" max="1"/>
@@ -30179,6 +30378,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -36078,6 +36278,33 @@
       <c r="F209" s="14" t="n"/>
       <c r="G209" s="14" t="n"/>
       <c r="H209" s="14" t="n"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>IS V01</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Generated from Reassembled OA Check; Wyoming OA not used as drafting source.</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Structural checks passed; visual render unavailable.</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -36411,7 +36638,6 @@
       <c r="D13" s="1" t="n"/>
       <c r="E13" s="1" t="n"/>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Regenerate Investment Services OA V02
</commit_message>
<xml_diff>
--- a/Project Rooms/Operating Agreements/working/Investment Services/Investment Services OA Process Control.xlsx
+++ b/Project Rooms/Operating Agreements/working/Investment Services/Investment Services OA Process Control.xlsx
@@ -6511,7 +6511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z201"/>
+  <dimension ref="A1:Z202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.75" customWidth="1" min="1" max="1"/>
@@ -12185,6 +12185,43 @@
         </is>
       </c>
     </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>IS V02</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>IS V02 - Investment Services OA Draft - from Reassembled OA Check.docx</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Reassembled OA Check / SYH framework; Wyoming OA date background only</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Regenerated draft applying title, working effective date, four equal members, and service-company purpose changes in summary and main body.</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Structural DOCX checks passed. Visual render not completed because converter path was unavailable.</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Open facts: confirm Secretary of State filing date, managers, tax classification, signer titles, Exhibit A contribution/unit detail.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
@@ -12199,7 +12236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z216"/>
+  <dimension ref="A1:Z220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -18253,6 +18290,134 @@
       <c r="F216" t="inlineStr">
         <is>
           <t>Applied in IS V01</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>IS-TITLE</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Entity title</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Investment Services drafts should title the entity Investment Services LLC, not Sell Your Home, LLC.</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Wes instruction 2026-06-16</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Applied in IS V02</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>IS-EQUAL-MEMBERS</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Member facts</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Members are Buy Your Home, LLC, Sell Your Home, LLC, Heritage Management LLC, and BYH 401K LLC, each at 25%.</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Wes instruction 2026-06-16</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Applied in IS V02</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>IS-SERVICE-PURPOSE</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Business purpose</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Investment Services LLC is not an investment company and is not limited to residential real estate investment; it provides services to other investment companies including management, signing authority, and buyer qualification services.</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Wes instruction 2026-06-16</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Applied in IS V02</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>IS-WYOMING-DATE-ONLY</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Source limitation</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Use the Wyoming OA only for the start/effective date unless Wes explicitly authorizes other use.</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Wes instruction 2026-06-16</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Applied in IS V02</t>
         </is>
       </c>
     </row>
@@ -24427,7 +24592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z203"/>
+  <dimension ref="A1:Z204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.25" customWidth="1" min="1" max="1"/>
@@ -30344,6 +30509,38 @@
         </is>
       </c>
     </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>IS-START-DATE-CONFIRM</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Effective date</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>V02 uses January 17, 2025 from the Wyoming OA file date/effective-date concept. Confirm the Secretary of State filing date before final use.</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Wes/records</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
@@ -30358,7 +30555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z210"/>
+  <dimension ref="A1:Z211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.75" customWidth="1" min="1" max="1"/>
@@ -36301,6 +36498,33 @@
         </is>
       </c>
       <c r="E210" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>IS V02</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Regenerated from Reassembled OA Check; Wyoming OA used only for date background.</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Structural checks passed; visual render unavailable.</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>

</xml_diff>

<commit_message>
Build Investment Services OA V03
</commit_message>
<xml_diff>
--- a/Project Rooms/Operating Agreements/working/Investment Services/Investment Services OA Process Control.xlsx
+++ b/Project Rooms/Operating Agreements/working/Investment Services/Investment Services OA Process Control.xlsx
@@ -181,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -228,6 +228,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6379,103 +6388,104 @@
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>Investment Services Operating Agreement Process Control Workbook</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Document and control the reusable process for creating an Investment Services LLC operating agreement from SYH / Jeff Watson source pieces, using a BYH-like process structure without copying BYH entity facts.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Current Source</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>SYH Simplified OA or Reassembled OA Check; Wyoming Investment Services OA is background/reference only unless Wes explicitly changes this rule.</t>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Reassembled OA Check from controlled local Simplified OA subfile stack; Teams/SharePoint is not refreshed unless Wes explicitly names a Teams file as a new source.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>Current Best Draft</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>Not built yet in this mode.</t>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>IS V03 - Investment Services OA Draft - from Reassembled OA Check.docx</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>Build Rule</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Do not build a new OA version until Wes explicitly says to build one.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>Future Filename Rule</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Future version filenames should start with the version identifier, e.g. IS V01 - Investment Services OA Draft ...</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>Source Lineage</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Preserve SYH/Jeff Watson source lineage; use green font for Investment Services additions/replacements unless Wes changes the rule.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Visual QA Limitation</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>DOCX render checks may be blocked locally by a missing converter executable; use structural XML checks if rendering is unavailable.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>Owner Review</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Legal, tax, authority, member-rights, and entity-specific assumptions require attorney/CPA review before final use.</t>
         </is>
@@ -6511,7 +6521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z202"/>
+  <dimension ref="A1:Z203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.75" customWidth="1" min="1" max="1"/>
@@ -6525,7 +6535,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>Version Log</t>
         </is>
@@ -6533,47 +6543,47 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="22" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="22" t="inlineStr">
         <is>
           <t>File Name</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="22" t="inlineStr">
         <is>
           <t>Source Used</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="22" t="inlineStr">
         <is>
           <t>Build Type</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="22" t="inlineStr">
         <is>
           <t>Purpose / Major Change</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="22" t="inlineStr">
         <is>
           <t>Known Issue Fixed</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="22" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="22" t="inlineStr">
         <is>
           <t>Comparison / Notes</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="22" t="inlineStr">
         <is>
           <t>Future Baseline?</t>
         </is>
@@ -12149,76 +12159,123 @@
       <c r="Z200" s="5" t="n"/>
     </row>
     <row r="201">
-      <c r="A201" t="inlineStr">
+      <c r="A201" s="18" t="inlineStr">
         <is>
           <t>IS V01</t>
         </is>
       </c>
-      <c r="B201" t="inlineStr">
+      <c r="B201" s="18" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="C201" t="inlineStr">
+      <c r="C201" s="18" t="inlineStr">
         <is>
           <t>IS V01 - Investment Services OA Draft - from Reassembled OA Check.docx</t>
         </is>
       </c>
-      <c r="D201" t="inlineStr">
+      <c r="D201" s="18" t="inlineStr">
         <is>
           <t>Reassembled OA Check / SYH framework</t>
         </is>
       </c>
-      <c r="E201" t="inlineStr">
+      <c r="E201" s="18" t="inlineStr">
         <is>
           <t>First Investment Services draft. Redlines SYH entity name to Investment Services LLC, strikes opening retirement-account member lines, inserts Investment Services member placeholder, marks Manager(s), tax classification, certification/signature, and Exhibit A as unconfirmed.</t>
         </is>
       </c>
-      <c r="F201" t="inlineStr">
+      <c r="F201" s="18" t="inlineStr">
         <is>
           <t>Structural DOCX checks passed. Visual render not completed because converter path was unavailable.</t>
         </is>
       </c>
-      <c r="G201" t="inlineStr">
+      <c r="G201" s="18" t="inlineStr">
         <is>
           <t>Open facts: members/ownership, managers, tax classification, effective date, signer titles, Exhibit A.</t>
         </is>
       </c>
     </row>
     <row r="202">
-      <c r="A202" t="inlineStr">
+      <c r="A202" s="18" t="inlineStr">
         <is>
           <t>IS V02</t>
         </is>
       </c>
-      <c r="B202" t="inlineStr">
+      <c r="B202" s="18" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="C202" t="inlineStr">
+      <c r="C202" s="18" t="inlineStr">
         <is>
           <t>IS V02 - Investment Services OA Draft - from Reassembled OA Check.docx</t>
         </is>
       </c>
-      <c r="D202" t="inlineStr">
+      <c r="D202" s="18" t="inlineStr">
         <is>
           <t>Reassembled OA Check / SYH framework; Wyoming OA date background only</t>
         </is>
       </c>
-      <c r="E202" t="inlineStr">
+      <c r="E202" s="18" t="inlineStr">
         <is>
           <t>Regenerated draft applying title, working effective date, four equal members, and service-company purpose changes in summary and main body.</t>
         </is>
       </c>
-      <c r="F202" t="inlineStr">
+      <c r="F202" s="18" t="inlineStr">
         <is>
           <t>Structural DOCX checks passed. Visual render not completed because converter path was unavailable.</t>
         </is>
       </c>
-      <c r="G202" t="inlineStr">
+      <c r="G202" s="18" t="inlineStr">
         <is>
           <t>Open facts: confirm Secretary of State filing date, managers, tax classification, signer titles, Exhibit A contribution/unit detail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="18" t="inlineStr">
+        <is>
+          <t>IS V03</t>
+        </is>
+      </c>
+      <c r="B203" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C203" s="18" t="inlineStr">
+        <is>
+          <t>IS V03 - Investment Services OA Draft - from Reassembled OA Check.docx</t>
+        </is>
+      </c>
+      <c r="D203" s="18" t="inlineStr">
+        <is>
+          <t>Fresh from current Reassembled OA Check; Wyoming OA date background only</t>
+        </is>
+      </c>
+      <c r="E203" s="18" t="inlineStr">
+        <is>
+          <t>Regenerated after the source stack gained the Drafting Legend and SYH source-level entity-manager language. Applies cumulative IS facts, adds agreement page/version footer, leaves Drafting Legend section footerless, and adds manager-review marker for the Investment Services-as-manager source clause.</t>
+        </is>
+      </c>
+      <c r="F203" s="18" t="inlineStr">
+        <is>
+          <t>Structural DOCX checks passed. LibreOffice PDF conversion passed at 27 pages; page-image QA unavailable in this environment.</t>
+        </is>
+      </c>
+      <c r="G203" s="18" t="inlineStr">
+        <is>
+          <t>Open facts: confirm Secretary of State filing date, managers, tax classification, signer titles, Exhibit A contribution/unit detail, and treatment of source entity-manager clause.</t>
+        </is>
+      </c>
+      <c r="H203" s="18" t="inlineStr">
+        <is>
+          <t>IS V03 notes</t>
+        </is>
+      </c>
+      <c r="I203" s="18" t="inlineStr">
+        <is>
+          <t>Yes - current working draft</t>
         </is>
       </c>
     </row>
@@ -12236,7 +12293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z220"/>
+  <dimension ref="A1:Z221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12250,7 +12307,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>Rule Register</t>
         </is>
@@ -12258,42 +12315,42 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="22" t="inlineStr">
         <is>
           <t>Rule ID</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="22" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="22" t="inlineStr">
         <is>
           <t>Rule / Instruction</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="22" t="inlineStr">
         <is>
           <t>Applies To</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="22" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="22" t="inlineStr">
         <is>
           <t>Build Impact</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="22" t="inlineStr">
         <is>
           <t>Verification</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="22" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -18230,194 +18287,226 @@
       <c r="H214" s="14" t="n"/>
     </row>
     <row r="215">
-      <c r="A215" t="inlineStr">
+      <c r="A215" s="18" t="inlineStr">
         <is>
           <t>IS-START-REASSEMBLED</t>
         </is>
       </c>
-      <c r="B215" t="inlineStr">
+      <c r="B215" s="18" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="C215" t="inlineStr">
+      <c r="C215" s="18" t="inlineStr">
         <is>
           <t>Source selection</t>
         </is>
       </c>
-      <c r="D215" t="inlineStr">
+      <c r="D215" s="18" t="inlineStr">
         <is>
           <t>All Investment Services drafts using the SYH/Simplified OA framework begin from the Reassembled OA Check unless Wes explicitly names another source.</t>
         </is>
       </c>
-      <c r="E215" t="inlineStr">
+      <c r="E215" s="18" t="inlineStr">
         <is>
           <t>Wes instruction 2026-06-16</t>
         </is>
       </c>
-      <c r="F215" t="inlineStr">
+      <c r="F215" s="18" t="inlineStr">
         <is>
           <t>Applied in IS V01</t>
         </is>
       </c>
     </row>
     <row r="216">
-      <c r="A216" t="inlineStr">
+      <c r="A216" s="18" t="inlineStr">
         <is>
           <t>IS-NO-WYOMING-SOURCE</t>
         </is>
       </c>
-      <c r="B216" t="inlineStr">
+      <c r="B216" s="18" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="C216" t="inlineStr">
+      <c r="C216" s="18" t="inlineStr">
         <is>
           <t>Source exclusion</t>
         </is>
       </c>
-      <c r="D216" t="inlineStr">
+      <c r="D216" s="18" t="inlineStr">
         <is>
           <t>Do not use the Wyoming Investment Services OA as the drafting source unless Wes explicitly changes that rule.</t>
         </is>
       </c>
-      <c r="E216" t="inlineStr">
+      <c r="E216" s="18" t="inlineStr">
         <is>
           <t>Wes instruction 2026-06-16</t>
         </is>
       </c>
-      <c r="F216" t="inlineStr">
+      <c r="F216" s="18" t="inlineStr">
         <is>
           <t>Applied in IS V01</t>
         </is>
       </c>
     </row>
     <row r="217">
-      <c r="A217" t="inlineStr">
+      <c r="A217" s="18" t="inlineStr">
         <is>
           <t>IS-TITLE</t>
         </is>
       </c>
-      <c r="B217" t="inlineStr">
+      <c r="B217" s="18" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="C217" t="inlineStr">
+      <c r="C217" s="18" t="inlineStr">
         <is>
           <t>Entity title</t>
         </is>
       </c>
-      <c r="D217" t="inlineStr">
+      <c r="D217" s="18" t="inlineStr">
         <is>
           <t>Investment Services drafts should title the entity Investment Services LLC, not Sell Your Home, LLC.</t>
         </is>
       </c>
-      <c r="E217" t="inlineStr">
+      <c r="E217" s="18" t="inlineStr">
         <is>
           <t>Wes instruction 2026-06-16</t>
         </is>
       </c>
-      <c r="F217" t="inlineStr">
+      <c r="F217" s="18" t="inlineStr">
         <is>
           <t>Applied in IS V02</t>
         </is>
       </c>
     </row>
     <row r="218">
-      <c r="A218" t="inlineStr">
+      <c r="A218" s="18" t="inlineStr">
         <is>
           <t>IS-EQUAL-MEMBERS</t>
         </is>
       </c>
-      <c r="B218" t="inlineStr">
+      <c r="B218" s="18" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="C218" t="inlineStr">
+      <c r="C218" s="18" t="inlineStr">
         <is>
           <t>Member facts</t>
         </is>
       </c>
-      <c r="D218" t="inlineStr">
+      <c r="D218" s="18" t="inlineStr">
         <is>
           <t>Members are Buy Your Home, LLC, Sell Your Home, LLC, Heritage Management LLC, and BYH 401K LLC, each at 25%.</t>
         </is>
       </c>
-      <c r="E218" t="inlineStr">
+      <c r="E218" s="18" t="inlineStr">
         <is>
           <t>Wes instruction 2026-06-16</t>
         </is>
       </c>
-      <c r="F218" t="inlineStr">
+      <c r="F218" s="18" t="inlineStr">
         <is>
           <t>Applied in IS V02</t>
         </is>
       </c>
     </row>
     <row r="219">
-      <c r="A219" t="inlineStr">
+      <c r="A219" s="18" t="inlineStr">
         <is>
           <t>IS-SERVICE-PURPOSE</t>
         </is>
       </c>
-      <c r="B219" t="inlineStr">
+      <c r="B219" s="18" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="C219" t="inlineStr">
+      <c r="C219" s="18" t="inlineStr">
         <is>
           <t>Business purpose</t>
         </is>
       </c>
-      <c r="D219" t="inlineStr">
+      <c r="D219" s="18" t="inlineStr">
         <is>
           <t>Investment Services LLC is not an investment company and is not limited to residential real estate investment; it provides services to other investment companies including management, signing authority, and buyer qualification services.</t>
         </is>
       </c>
-      <c r="E219" t="inlineStr">
+      <c r="E219" s="18" t="inlineStr">
         <is>
           <t>Wes instruction 2026-06-16</t>
         </is>
       </c>
-      <c r="F219" t="inlineStr">
+      <c r="F219" s="18" t="inlineStr">
         <is>
           <t>Applied in IS V02</t>
         </is>
       </c>
     </row>
     <row r="220">
-      <c r="A220" t="inlineStr">
+      <c r="A220" s="18" t="inlineStr">
         <is>
           <t>IS-WYOMING-DATE-ONLY</t>
         </is>
       </c>
-      <c r="B220" t="inlineStr">
+      <c r="B220" s="18" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="C220" t="inlineStr">
+      <c r="C220" s="18" t="inlineStr">
         <is>
           <t>Source limitation</t>
         </is>
       </c>
-      <c r="D220" t="inlineStr">
+      <c r="D220" s="18" t="inlineStr">
         <is>
           <t>Use the Wyoming OA only for the start/effective date unless Wes explicitly authorizes other use.</t>
         </is>
       </c>
-      <c r="E220" t="inlineStr">
+      <c r="E220" s="18" t="inlineStr">
         <is>
           <t>Wes instruction 2026-06-16</t>
         </is>
       </c>
-      <c r="F220" t="inlineStr">
+      <c r="F220" s="18" t="inlineStr">
         <is>
           <t>Applied in IS V02</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="18" t="inlineStr">
+        <is>
+          <t>IS-NO-TEAMS-SOURCE</t>
+        </is>
+      </c>
+      <c r="B221" s="18" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C221" s="18" t="inlineStr">
+        <is>
+          <t>Source limitation</t>
+        </is>
+      </c>
+      <c r="D221" s="18" t="inlineStr">
+        <is>
+          <t>Do not refresh or pull the Simplified OA from Teams/SharePoint before a derivative build merely because a new draft is requested; Teams is final delivery/archive unless Wes explicitly identifies a Teams file as a new source.</t>
+        </is>
+      </c>
+      <c r="E221" s="18" t="inlineStr">
+        <is>
+          <t>Wes instruction / project-room rule</t>
+        </is>
+      </c>
+      <c r="F221" s="18" t="inlineStr">
+        <is>
+          <t>Applied in IS V03</t>
         </is>
       </c>
     </row>
@@ -24592,7 +24681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z204"/>
+  <dimension ref="A1:Z205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.25" customWidth="1" min="1" max="1"/>
@@ -24606,7 +24695,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>Open Issues</t>
         </is>
@@ -24614,42 +24703,42 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="22" t="inlineStr">
         <is>
           <t>Issue ID</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="22" t="inlineStr">
         <is>
           <t>Area</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="22" t="inlineStr">
         <is>
           <t>Question / Risk</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="22" t="inlineStr">
         <is>
           <t>Current Assumption</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="22" t="inlineStr">
         <is>
           <t>Owner / Reviewer</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="22" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="22" t="inlineStr">
         <is>
           <t>Needed Before Final?</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="22" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -24696,22 +24785,22 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Wes / Codex</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed for current builds</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>Before first draft</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>Teams refresh may be needed.</t>
+          <t>Use current local Reassembled OA Check. Do not refresh from Teams unless Wes explicitly identifies a Teams file as a new source.</t>
         </is>
       </c>
       <c r="I4" s="5" t="n"/>
@@ -30414,130 +30503,172 @@
       <c r="Z200" s="5" t="n"/>
     </row>
     <row r="201">
-      <c r="A201" t="inlineStr">
+      <c r="A201" s="18" t="inlineStr">
         <is>
           <t>IS-MEMBERS</t>
         </is>
       </c>
-      <c r="B201" t="inlineStr">
+      <c r="B201" s="18" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="C201" t="inlineStr">
+      <c r="C201" s="18" t="inlineStr">
         <is>
           <t>Member facts</t>
         </is>
       </c>
-      <c r="D201" t="inlineStr">
+      <c r="D201" s="18" t="inlineStr">
         <is>
           <t>Confirm current Investment Services LLC member(s), ownership units or percentages, contributions, and whether any retirement-account ownership exists.</t>
         </is>
       </c>
-      <c r="E201" t="inlineStr">
+      <c r="E201" s="18" t="inlineStr">
         <is>
           <t>Wes/records</t>
         </is>
       </c>
-      <c r="F201" t="inlineStr">
+      <c r="F201" s="18" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
     <row r="202">
-      <c r="A202" t="inlineStr">
+      <c r="A202" s="18" t="inlineStr">
         <is>
           <t>IS-MANAGERS</t>
         </is>
       </c>
-      <c r="B202" t="inlineStr">
+      <c r="B202" s="18" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="C202" t="inlineStr">
+      <c r="C202" s="18" t="inlineStr">
         <is>
           <t>Manager facts</t>
         </is>
       </c>
-      <c r="D202" t="inlineStr">
+      <c r="D202" s="18" t="inlineStr">
         <is>
           <t>Confirm current Investment Services LLC manager(s) and signer titles.</t>
         </is>
       </c>
-      <c r="E202" t="inlineStr">
+      <c r="E202" s="18" t="inlineStr">
         <is>
           <t>Wes/records</t>
         </is>
       </c>
-      <c r="F202" t="inlineStr">
+      <c r="F202" s="18" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
     <row r="203">
-      <c r="A203" t="inlineStr">
+      <c r="A203" s="18" t="inlineStr">
         <is>
           <t>IS-TAX</t>
         </is>
       </c>
-      <c r="B203" t="inlineStr">
+      <c r="B203" s="18" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="C203" t="inlineStr">
+      <c r="C203" s="18" t="inlineStr">
         <is>
           <t>Tax classification</t>
         </is>
       </c>
-      <c r="D203" t="inlineStr">
+      <c r="D203" s="18" t="inlineStr">
         <is>
           <t>Confirm tax classification before finalizing pass-through, S-corp, IRA, UBTI/UDFI, or retirement-account provisions.</t>
         </is>
       </c>
-      <c r="E203" t="inlineStr">
+      <c r="E203" s="18" t="inlineStr">
         <is>
           <t>CPA/attorney</t>
         </is>
       </c>
-      <c r="F203" t="inlineStr">
+      <c r="F203" s="18" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
     <row r="204">
-      <c r="A204" t="inlineStr">
+      <c r="A204" s="18" t="inlineStr">
         <is>
           <t>IS-START-DATE-CONFIRM</t>
         </is>
       </c>
-      <c r="B204" t="inlineStr">
+      <c r="B204" s="18" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="C204" t="inlineStr">
+      <c r="C204" s="18" t="inlineStr">
         <is>
           <t>Effective date</t>
         </is>
       </c>
-      <c r="D204" t="inlineStr">
+      <c r="D204" s="18" t="inlineStr">
         <is>
           <t>V02 uses January 17, 2025 from the Wyoming OA file date/effective-date concept. Confirm the Secretary of State filing date before final use.</t>
         </is>
       </c>
-      <c r="E204" t="inlineStr">
+      <c r="E204" s="18" t="inlineStr">
         <is>
           <t>Wes/records</t>
         </is>
       </c>
-      <c r="F204" t="inlineStr">
+      <c r="F204" s="18" t="inlineStr">
         <is>
           <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="18" t="inlineStr">
+        <is>
+          <t>IS-ENTITY-MANAGER-CLAUSE</t>
+        </is>
+      </c>
+      <c r="B205" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C205" s="18" t="inlineStr">
+        <is>
+          <t>Manager language</t>
+        </is>
+      </c>
+      <c r="D205" s="18" t="inlineStr">
+        <is>
+          <t>Confirm how the SYH source clause allowing Investment Services LLC to serve as Manager should be handled in Investment Services LLC's own OA.</t>
+        </is>
+      </c>
+      <c r="E205" s="18" t="inlineStr">
+        <is>
+          <t>Wes/attorney</t>
+        </is>
+      </c>
+      <c r="F205" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G205" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H205" s="18" t="inlineStr">
+        <is>
+          <t>V03 adds a green review marker rather than treating the clause as final.</t>
         </is>
       </c>
     </row>
@@ -30555,7 +30686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z211"/>
+  <dimension ref="A1:Z212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.75" customWidth="1" min="1" max="1"/>
@@ -30569,7 +30700,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>Build Checklist</t>
         </is>
@@ -30577,42 +30708,42 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="22" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="22" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="22" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="22" t="inlineStr">
         <is>
           <t>Required?</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="22" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="22" t="inlineStr">
         <is>
           <t>Evidence / Output</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="22" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="22" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -30657,10 +30788,14 @@
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Pending for first build</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="n"/>
+          <t>Complete for IS V03</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>Wes said go after defining Run OA in IS mode.</t>
+        </is>
+      </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
           <t>Wes</t>
@@ -30769,10 +30904,14 @@
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Pending for first build</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="n"/>
+          <t>Complete for IS V03</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Used Reassembled OA Check; Teams not refreshed; Wyoming OA date background only.</t>
+        </is>
+      </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
           <t>Codex/Wes</t>
@@ -30823,10 +30962,14 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="n"/>
+          <t>Partially complete for IS V03</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>Known facts applied; manager, tax, signer, Exhibit A details remain open.</t>
+        </is>
+      </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Wes/Codex</t>
@@ -30935,10 +31078,14 @@
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="n"/>
+          <t>Complete for IS V03</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>IS V03 DOCX generated.</t>
+        </is>
+      </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
           <t>Codex</t>
@@ -30989,10 +31136,14 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="n"/>
+          <t>Complete with limitation for IS V03</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Structural checks passed; LibreOffice PDF conversion passed at 27 pages; page-image QA unavailable.</t>
+        </is>
+      </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
           <t>Codex</t>
@@ -31043,10 +31194,14 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="n"/>
+          <t>Complete for IS V03</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Notes, source inventory, README, and workbook updated.</t>
+        </is>
+      </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
           <t>Codex</t>
@@ -36477,54 +36632,81 @@
       <c r="H209" s="14" t="n"/>
     </row>
     <row r="210">
-      <c r="A210" t="inlineStr">
+      <c r="A210" s="18" t="inlineStr">
         <is>
           <t>IS V01</t>
         </is>
       </c>
-      <c r="B210" t="inlineStr">
+      <c r="B210" s="18" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="C210" t="inlineStr">
+      <c r="C210" s="18" t="inlineStr">
         <is>
           <t>Generated from Reassembled OA Check; Wyoming OA not used as drafting source.</t>
         </is>
       </c>
-      <c r="D210" t="inlineStr">
+      <c r="D210" s="18" t="inlineStr">
         <is>
           <t>Structural checks passed; visual render unavailable.</t>
         </is>
       </c>
-      <c r="E210" t="inlineStr">
+      <c r="E210" s="18" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="211">
-      <c r="A211" t="inlineStr">
+      <c r="A211" s="18" t="inlineStr">
         <is>
           <t>IS V02</t>
         </is>
       </c>
-      <c r="B211" t="inlineStr">
+      <c r="B211" s="18" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="C211" t="inlineStr">
+      <c r="C211" s="18" t="inlineStr">
         <is>
           <t>Regenerated from Reassembled OA Check; Wyoming OA used only for date background.</t>
         </is>
       </c>
-      <c r="D211" t="inlineStr">
+      <c r="D211" s="18" t="inlineStr">
         <is>
           <t>Structural checks passed; visual render unavailable.</t>
         </is>
       </c>
-      <c r="E211" t="inlineStr">
+      <c r="E211" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="18" t="inlineStr">
+        <is>
+          <t>IS V03</t>
+        </is>
+      </c>
+      <c r="B212" s="18" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="C212" s="18" t="inlineStr">
+        <is>
+          <t>Generated from current Reassembled OA Check with Drafting Legend source stack.</t>
+        </is>
+      </c>
+      <c r="D212" s="18" t="inlineStr">
+        <is>
+          <t>Structural checks passed; PDF conversion passed at 27 pages; page-image QA unavailable.</t>
+        </is>
+      </c>
+      <c r="E212" s="18" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>

</xml_diff>

<commit_message>
Build Investment Services OA V04 adjustments
</commit_message>
<xml_diff>
--- a/Project Rooms/Operating Agreements/working/Investment Services/Investment Services OA Process Control.xlsx
+++ b/Project Rooms/Operating Agreements/working/Investment Services/Investment Services OA Process Control.xlsx
@@ -6394,7 +6394,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="21" t="inlineStr">
         <is>
@@ -6427,7 +6426,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>IS V03 - Investment Services OA Draft - from Reassembled OA Check.docx</t>
+          <t>IS V04 - Investment Services OA Draft - from Reassembled OA Check.docx</t>
         </is>
       </c>
     </row>
@@ -6521,7 +6520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z203"/>
+  <dimension ref="A1:Z204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.75" customWidth="1" min="1" max="1"/>
@@ -12279,6 +12278,53 @@
         </is>
       </c>
     </row>
+    <row r="204">
+      <c r="A204" s="18" t="inlineStr">
+        <is>
+          <t>IS V04</t>
+        </is>
+      </c>
+      <c r="B204" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C204" s="18" t="inlineStr">
+        <is>
+          <t>IS V04 - Investment Services OA Draft - from Reassembled OA Check.docx</t>
+        </is>
+      </c>
+      <c r="D204" s="18" t="inlineStr">
+        <is>
+          <t>Fresh from current Reassembled OA Check; Wyoming OA date background only</t>
+        </is>
+      </c>
+      <c r="E204" s="18" t="inlineStr">
+        <is>
+          <t>Regenerated using Wes V04 adjustments: minimum practical redlines, Article 1 negative phrase omitted, Entity Manager Authority omitted, 5.1(b)(xi) retained unstruck, 9.1/9.2/9.6 struck, and Investment Services removed from certification manager block.</t>
+        </is>
+      </c>
+      <c r="F204" s="18" t="inlineStr">
+        <is>
+          <t>Structural DOCX checks passed. LibreOffice PDF conversion passed at 26 pages; packaged page-image rendering timed out in this environment.</t>
+        </is>
+      </c>
+      <c r="G204" s="18" t="inlineStr">
+        <is>
+          <t>Open facts: confirm Secretary of State filing date, managers, tax classification, signer titles, and Exhibit A contribution/unit detail.</t>
+        </is>
+      </c>
+      <c r="H204" s="18" t="inlineStr">
+        <is>
+          <t>IS V04 notes</t>
+        </is>
+      </c>
+      <c r="I204" s="18" t="inlineStr">
+        <is>
+          <t>Yes - current working draft</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
@@ -12293,7 +12339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z221"/>
+  <dimension ref="A1:Z227"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12313,7 +12359,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="22" t="inlineStr">
         <is>
@@ -18507,6 +18552,198 @@
       <c r="F221" s="18" t="inlineStr">
         <is>
           <t>Applied in IS V03</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="18" t="inlineStr">
+        <is>
+          <t>IS-MIN-CHANGE</t>
+        </is>
+      </c>
+      <c r="B222" s="18" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C222" s="18" t="inlineStr">
+        <is>
+          <t>Drafting method</t>
+        </is>
+      </c>
+      <c r="D222" s="18" t="inlineStr">
+        <is>
+          <t>Make the minimum practical redline changes needed; do not replace a whole paragraph when targeted word or phrase replacements will do.</t>
+        </is>
+      </c>
+      <c r="E222" s="18" t="inlineStr">
+        <is>
+          <t>Wes instruction 2026-06-16</t>
+        </is>
+      </c>
+      <c r="F222" s="18" t="inlineStr">
+        <is>
+          <t>Applied in IS V04</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="18" t="inlineStr">
+        <is>
+          <t>IS-ARTICLE1-PURPOSE</t>
+        </is>
+      </c>
+      <c r="B223" s="18" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C223" s="18" t="inlineStr">
+        <is>
+          <t>Business purpose</t>
+        </is>
+      </c>
+      <c r="D223" s="18" t="inlineStr">
+        <is>
+          <t>In summary and Article 1 counterpart, omit the added phrase Business is not limited to residential real estate investment.</t>
+        </is>
+      </c>
+      <c r="E223" s="18" t="inlineStr">
+        <is>
+          <t>Wes instruction 2026-06-16</t>
+        </is>
+      </c>
+      <c r="F223" s="18" t="inlineStr">
+        <is>
+          <t>Applied in IS V04</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="18" t="inlineStr">
+        <is>
+          <t>IS-OMIT-ENTITY-MANAGER</t>
+        </is>
+      </c>
+      <c r="B224" s="18" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C224" s="18" t="inlineStr">
+        <is>
+          <t>Manager language</t>
+        </is>
+      </c>
+      <c r="D224" s="18" t="inlineStr">
+        <is>
+          <t>Leave out the Entity Manager Authority paragraph and related manager-review note from Investment Services LLC own OA.</t>
+        </is>
+      </c>
+      <c r="E224" s="18" t="inlineStr">
+        <is>
+          <t>Wes instruction 2026-06-16</t>
+        </is>
+      </c>
+      <c r="F224" s="18" t="inlineStr">
+        <is>
+          <t>Applied in IS V04</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="18" t="inlineStr">
+        <is>
+          <t>IS-RETAIN-5-1-B-XI</t>
+        </is>
+      </c>
+      <c r="B225" s="18" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C225" s="18" t="inlineStr">
+        <is>
+          <t>Article 5</t>
+        </is>
+      </c>
+      <c r="D225" s="18" t="inlineStr">
+        <is>
+          <t>Keep Section 5.1(b)(xi) operative and unstruck.</t>
+        </is>
+      </c>
+      <c r="E225" s="18" t="inlineStr">
+        <is>
+          <t>Wes instruction 2026-06-16</t>
+        </is>
+      </c>
+      <c r="F225" s="18" t="inlineStr">
+        <is>
+          <t>Applied in IS V04</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="18" t="inlineStr">
+        <is>
+          <t>IS-STRIKE-9-1-9-2-9-6</t>
+        </is>
+      </c>
+      <c r="B226" s="18" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C226" s="18" t="inlineStr">
+        <is>
+          <t>Article 9</t>
+        </is>
+      </c>
+      <c r="D226" s="18" t="inlineStr">
+        <is>
+          <t>Strike Sections 9.1, 9.2, and 9.6 while preserving paragraph positions.</t>
+        </is>
+      </c>
+      <c r="E226" s="18" t="inlineStr">
+        <is>
+          <t>Wes instruction 2026-06-16</t>
+        </is>
+      </c>
+      <c r="F226" s="18" t="inlineStr">
+        <is>
+          <t>Applied in IS V04</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="18" t="inlineStr">
+        <is>
+          <t>IS-CERT-NO-IS-MANAGER</t>
+        </is>
+      </c>
+      <c r="B227" s="18" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C227" s="18" t="inlineStr">
+        <is>
+          <t>Certification</t>
+        </is>
+      </c>
+      <c r="D227" s="18" t="inlineStr">
+        <is>
+          <t>Remove Investment Services LLC from the certification manager/signature block.</t>
+        </is>
+      </c>
+      <c r="E227" s="18" t="inlineStr">
+        <is>
+          <t>Wes instruction 2026-06-16</t>
+        </is>
+      </c>
+      <c r="F227" s="18" t="inlineStr">
+        <is>
+          <t>Applied in IS V04</t>
         </is>
       </c>
     </row>
@@ -24701,7 +24938,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="22" t="inlineStr">
         <is>
@@ -30658,17 +30894,17 @@
       </c>
       <c r="F205" s="18" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed for current build</t>
         </is>
       </c>
       <c r="G205" s="18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H205" s="18" t="inlineStr">
         <is>
-          <t>V03 adds a green review marker rather than treating the clause as final.</t>
+          <t>V04 omits the source Entity Manager Authority clause from Investment Services LLC own OA.</t>
         </is>
       </c>
     </row>
@@ -30686,7 +30922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z212"/>
+  <dimension ref="A1:Z213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.75" customWidth="1" min="1" max="1"/>
@@ -30788,12 +31024,12 @@
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Complete for IS V03</t>
+          <t>Complete for IS V04</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>Wes said go after defining Run OA in IS mode.</t>
+          <t>Wes gave adjustment list and said go.</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
@@ -30904,7 +31140,7 @@
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Complete for IS V03</t>
+          <t>Complete for IS V04</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
@@ -30962,12 +31198,12 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>Partially complete for IS V03</t>
+          <t>Partially complete for IS V04</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>Known facts applied; manager, tax, signer, Exhibit A details remain open.</t>
+          <t>Known facts and V04 adjustments applied; manager, tax, signer, Exhibit A details remain open.</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
@@ -31078,12 +31314,12 @@
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>Complete for IS V03</t>
+          <t>Complete for IS V04</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>IS V03 DOCX generated.</t>
+          <t>IS V04 DOCX generated.</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
@@ -31136,12 +31372,12 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Complete with limitation for IS V03</t>
+          <t>Complete with limitation for IS V04</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Structural checks passed; LibreOffice PDF conversion passed at 27 pages; page-image QA unavailable.</t>
+          <t>Structural checks passed; LibreOffice PDF conversion passed at 26 pages; packaged page-image rendering timed out.</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
@@ -31194,12 +31430,12 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Complete for IS V03</t>
+          <t>Complete for IS V04</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Notes, source inventory, README, and workbook updated.</t>
+          <t>Notes, source inventory, README, rules, and workbook updated.</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
@@ -36707,6 +36943,33 @@
         </is>
       </c>
       <c r="E212" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="18" t="inlineStr">
+        <is>
+          <t>IS V04</t>
+        </is>
+      </c>
+      <c r="B213" s="18" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="C213" s="18" t="inlineStr">
+        <is>
+          <t>Generated from current Reassembled OA Check with V04 adjustment list.</t>
+        </is>
+      </c>
+      <c r="D213" s="18" t="inlineStr">
+        <is>
+          <t>Structural checks passed; PDF conversion passed at 26 pages; packaged page-image rendering timed out.</t>
+        </is>
+      </c>
+      <c r="E213" s="18" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>

</xml_diff>

<commit_message>
Build Investment Services OA V05
</commit_message>
<xml_diff>
--- a/Project Rooms/Operating Agreements/working/Investment Services/Investment Services OA Process Control.xlsx
+++ b/Project Rooms/Operating Agreements/working/Investment Services/Investment Services OA Process Control.xlsx
@@ -6394,6 +6394,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="21" t="inlineStr">
         <is>
@@ -6426,7 +6427,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>IS V04 - Investment Services OA Draft - from Reassembled OA Check.docx</t>
+          <t>IS V05 - Investment Services OA Draft - from Reassembled OA Check.docx</t>
         </is>
       </c>
     </row>
@@ -6520,7 +6521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z204"/>
+  <dimension ref="A1:Z205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.75" customWidth="1" min="1" max="1"/>
@@ -6540,7 +6541,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="22" t="inlineStr">
         <is>
@@ -12322,6 +12322,53 @@
       <c r="I204" s="18" t="inlineStr">
         <is>
           <t>Yes - current working draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>IS V05</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>IS V05 - Investment Services OA Draft - from Reassembled OA Check.docx</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Reassembled OA Check from accepted-build Simplified OA stack</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Fresh cumulative</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Regenerated Investment Services draft from current Reassembled OA Check after accepted-build stack refresh; carries forward V04 rules and replaces SYH Joshua Kennedy manager language with Investment Services [UNCONFIRMED Manager(s)] placeholder.</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Prevents SYH current-manager/source-stack language from being treated as Investment Services manager fact.</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Current working draft</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>IS V05 - Investment Services OA Draft Notes.md</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -30942,7 +30989,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="22" t="inlineStr">
         <is>
@@ -31024,12 +31070,12 @@
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Complete for IS V04</t>
+          <t>Complete for IS V05</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>Wes gave adjustment list and said go.</t>
+          <t>Wes said switch to Investment Services mode and give me a new build.</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
@@ -31372,12 +31418,12 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Complete with limitation for IS V04</t>
+          <t>Complete for IS V05</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Structural checks passed; LibreOffice PDF conversion passed at 26 pages; packaged page-image rendering timed out.</t>
+          <t>LibreOffice PDF conversion passed at 26 pages; PDF page images rendered and visually checked.</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Rebuild Investment Services OA V06
</commit_message>
<xml_diff>
--- a/Project Rooms/Operating Agreements/working/Investment Services/Investment Services OA Process Control.xlsx
+++ b/Project Rooms/Operating Agreements/working/Investment Services/Investment Services OA Process Control.xlsx
@@ -486,6 +486,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -718,7 +719,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>[UNCONFIRMED]</t>
+          <t>Buy Your Home, LLC</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -733,7 +734,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Needs Wes/source confirmation</t>
+          <t>Wes instruction</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -743,7 +744,7 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Do not copy BYH trust facts.</t>
+          <t>V06 uses 25 units / 25% working interest.</t>
         </is>
       </c>
       <c r="H7" s="5" t="n"/>
@@ -774,12 +775,12 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>[UNCONFIRMED]</t>
+          <t>Sell Your Home, LLC</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>No/TBD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -789,7 +790,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Needs Wes/source confirmation</t>
+          <t>Wes instruction</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -799,7 +800,7 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>May be blank if single-member.</t>
+          <t>V06 uses 25 units / 25% working interest.</t>
         </is>
       </c>
       <c r="H8" s="5" t="n"/>
@@ -1159,13 +1160,41 @@
       <c r="Z14" s="5" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="n"/>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="6" t="n"/>
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Member 3</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Heritage Management LLC</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Article 2 / Exhibit A / certification</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Wes instruction</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>V06 uses 25 units / 25% working interest.</t>
+        </is>
+      </c>
       <c r="H15" s="5" t="n"/>
       <c r="I15" s="5" t="n"/>
       <c r="J15" s="5" t="n"/>
@@ -1187,13 +1216,41 @@
       <c r="Z15" s="5" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Member 4</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>BYH 401K LLC</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Article 2 / Exhibit A / certification</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Wes instruction</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>V06 uses 25 units / 25% working interest.</t>
+        </is>
+      </c>
       <c r="H16" s="5" t="n"/>
       <c r="I16" s="5" t="n"/>
       <c r="J16" s="5" t="n"/>
@@ -1215,13 +1272,41 @@
       <c r="Z16" s="5" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Current Manager(s)</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Joshua Kennedy</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Article 5 / certification</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Wes confirmation</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Confirmed by Wes for V06 unless changed.</t>
+        </is>
+      </c>
       <c r="H17" s="5" t="n"/>
       <c r="I17" s="5" t="n"/>
       <c r="J17" s="5" t="n"/>
@@ -1243,13 +1328,41 @@
       <c r="Z17" s="5" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Membership percentages / units</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Each of four Members holds 25 units / 25%</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Opening / Article 2 / Exhibit A</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Wes instruction</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Address/email details remain TBD.</t>
+        </is>
+      </c>
       <c r="H18" s="5" t="n"/>
       <c r="I18" s="5" t="n"/>
       <c r="J18" s="5" t="n"/>
@@ -6427,7 +6540,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>IS V05 - Investment Services OA Draft - from Reassembled OA Check.docx</t>
+          <t>IS V06 - Investment Services OA Draft - from Reassembled OA Check.docx</t>
         </is>
       </c>
     </row>
@@ -6541,6 +6654,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="22" t="inlineStr">
         <is>
@@ -6670,15 +6784,51 @@
       <c r="Z4" s="5" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n"/>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>IS V06</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>IS V06 - Investment Services OA Draft - from Reassembled OA Check.docx</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Refreshed Reassembled OA Check from accepted Simplified OA build copy</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Fresh cumulative</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Confirmed Joshua Kennedy as current Manager; clean certification blocks; Exhibit A four 25-unit Members; retained V04 strike/unstrike rules.</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Removed placeholder manager, old IRA certification blocks, and old SYH Exhibit A table.</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Current working draft</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Structural checks passed; LibreOffice render passed at 27 pages with key-page visual checks.</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="J5" s="5" t="n"/>
       <c r="K5" s="5" t="n"/>
       <c r="L5" s="5" t="n"/>
@@ -12358,7 +12508,7 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>Current working draft</t>
+          <t>Prior / superseded by IS V06</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
@@ -12368,7 +12518,7 @@
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -12406,6 +12556,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="22" t="inlineStr">
         <is>
@@ -12947,14 +13098,46 @@
       <c r="Z11" s="5" t="n"/>
     </row>
     <row r="12" ht="25.5" customHeight="1">
-      <c r="A12" s="9" t="n"/>
-      <c r="B12" s="9" t="n"/>
-      <c r="C12" s="9" t="n"/>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="9" t="n"/>
-      <c r="F12" s="9" t="n"/>
-      <c r="G12" s="9" t="n"/>
-      <c r="H12" s="9" t="n"/>
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>IS-R-012</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Confirmed Facts</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Joshua Kennedy is the confirmed current Manager for Investment Services drafts unless Wes later changes that fact; certification and Exhibit A should use clean Investment Services-specific blocks, not old SYH/IRA blocks.</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Investment Services builds</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Controls Article 5, certification, and Exhibit A output</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Check Article 5, certification page, and Exhibit A in each build</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Added for IS V06 after Wes confirmed Joshua Kennedy as Manager.</t>
+        </is>
+      </c>
       <c r="I12" s="5" t="n"/>
       <c r="J12" s="5" t="n"/>
       <c r="K12" s="5" t="n"/>
@@ -24985,6 +25168,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="22" t="inlineStr">
         <is>
@@ -25123,7 +25307,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>[UNCONFIRMED]</t>
+          <t>Four Members confirmed: Buy Your Home, LLC; Sell Your Home, LLC; Heritage Management LLC; BYH 401K LLC, equal 25% / 25 units.</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -25133,7 +25317,7 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Partially closed</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -25143,7 +25327,7 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>Do not copy BYH trust facts.</t>
+          <t>Address/email and contribution details remain open before final.</t>
         </is>
       </c>
       <c r="I5" s="5" t="n"/>
@@ -25183,7 +25367,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>[UNCONFIRMED]</t>
+          <t>Joshua Kennedy confirmed as current Manager.</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -25193,7 +25377,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed for current draft</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -25203,7 +25387,7 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Do not copy BYH manager list by default.</t>
+          <t>Reopen if Wes adds another Manager or changes manager authority.</t>
         </is>
       </c>
       <c r="I6" s="5" t="n"/>
@@ -31070,12 +31254,12 @@
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Complete for IS V05</t>
+          <t>Complete for IS V06</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>Wes said switch to Investment Services mode and give me a new build.</t>
+          <t>Wes said see changes, rebuild stack, and create another draft.</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
@@ -31186,12 +31370,12 @@
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Complete for IS V04</t>
+          <t>Complete for IS V06</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Used Reassembled OA Check; Teams not refreshed; Wyoming OA date background only.</t>
+          <t>Used refreshed accepted-build Reassembled OA Check; Wyoming OA date background only.</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
@@ -31244,12 +31428,12 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>Partially complete for IS V04</t>
+          <t>Partially complete for IS V06</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>Known facts and V04 adjustments applied; manager, tax, signer, Exhibit A details remain open.</t>
+          <t>Members, equal units, and Joshua Manager applied; tax, date confirmation, signer titles, and address/email details remain open.</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Restore two-column OA certification layout
</commit_message>
<xml_diff>
--- a/Project Rooms/Operating Agreements/working/Investment Services/Investment Services OA Process Control.xlsx
+++ b/Project Rooms/Operating Agreements/working/Investment Services/Investment Services OA Process Control.xlsx
@@ -486,7 +486,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -6507,7 +6506,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="21" t="inlineStr">
         <is>
@@ -6654,7 +6652,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="22" t="inlineStr">
         <is>
@@ -13158,14 +13155,46 @@
       <c r="Z12" s="5" t="n"/>
     </row>
     <row r="13" ht="25.5" customHeight="1">
-      <c r="A13" s="9" t="n"/>
-      <c r="B13" s="9" t="n"/>
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="9" t="n"/>
-      <c r="E13" s="9" t="n"/>
-      <c r="F13" s="9" t="n"/>
-      <c r="G13" s="9" t="n"/>
-      <c r="H13" s="9" t="n"/>
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>IS-R-013</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Certification Layout</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Preserve the Simplified OA two-column certification-table approach where practical while replacing historical signer text with current Investment Services signer blocks.</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Investment Services certification pages</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Controls signing-page layout in review drafts and final candidates</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>Render certification page and verify two-column table layout</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>Added after Wes asked to restore the two-column certification approach.</t>
+        </is>
+      </c>
       <c r="I13" s="5" t="n"/>
       <c r="J13" s="5" t="n"/>
       <c r="K13" s="5" t="n"/>
@@ -25168,7 +25197,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="22" t="inlineStr">
         <is>
@@ -31698,14 +31726,46 @@
       <c r="Z11" s="5" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="n"/>
-      <c r="B12" s="9" t="n"/>
-      <c r="C12" s="9" t="n"/>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="9" t="n"/>
-      <c r="F12" s="9" t="n"/>
-      <c r="G12" s="9" t="n"/>
-      <c r="H12" s="9" t="n"/>
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Layout check</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Verify certification page uses two-column signing table where practical.</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Complete for IS V06</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Rendered certification page shows a one-page two-column signing table.</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Rule IS-R-013.</t>
+        </is>
+      </c>
       <c r="I12" s="5" t="n"/>
       <c r="J12" s="5" t="n"/>
       <c r="K12" s="5" t="n"/>

</xml_diff>

<commit_message>
Add Investment Services member signer names
</commit_message>
<xml_diff>
--- a/Project Rooms/Operating Agreements/working/Investment Services/Investment Services OA Process Control.xlsx
+++ b/Project Rooms/Operating Agreements/working/Investment Services/Investment Services OA Process Control.xlsx
@@ -486,6 +486,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -1383,13 +1384,41 @@
       <c r="Z18" s="5" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n"/>
-      <c r="B19" s="5" t="n"/>
-      <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="n"/>
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Member certification printed names</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Buy Your Home, LLC - Wesley Dale Browning; Sell Your Home, LLC - Joshua Kennedy; Heritage Management LLC - Wesley Dale Browning; BYH 401K LLC - Wesley Dale Browning.</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Certification page</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Wes instruction</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Used in two-column member signature table.</t>
+        </is>
+      </c>
       <c r="H19" s="5" t="n"/>
       <c r="I19" s="5" t="n"/>
       <c r="J19" s="5" t="n"/>
@@ -13215,14 +13244,46 @@
       <c r="Z13" s="5" t="n"/>
     </row>
     <row r="14" ht="25.5" customHeight="1">
-      <c r="A14" s="9" t="n"/>
-      <c r="B14" s="9" t="n"/>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="9" t="n"/>
-      <c r="E14" s="9" t="n"/>
-      <c r="F14" s="9" t="n"/>
-      <c r="G14" s="9" t="n"/>
-      <c r="H14" s="9" t="n"/>
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>IS-R-014</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Signature Blocks</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Member certification printed-name lines use Wesley Dale Browning for Buy Your Home, LLC, Heritage Management LLC, and BYH 401K LLC, and Joshua Kennedy for Sell Your Home, LLC.</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Investment Services certification pages</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Controls member signature block printed-name text</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>Check certification table printed-name lines</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>Added from Wes instruction.</t>
+        </is>
+      </c>
       <c r="I14" s="5" t="n"/>
       <c r="J14" s="5" t="n"/>
       <c r="K14" s="5" t="n"/>

</xml_diff>